<commit_message>
chore(outputs): crude family re-run folded at the TEN-reconciled basis — TEN range re-anchors 26.6/45.0 -> 25.2/42.0, point == family max again
The fold the containment-guard entry scheduled: the §9.10 sidecar's EV panel
re-anchors to the reconciled TEN balance sheet (Set A +42.0 == the live point
EV; every other crude name byte-identical), then the surface regenerates at
clean stamp 1a9e7b2. Delta 0 material / 0 new / 0 inputs changed; suite 590
green (containment + WO1-F1 stamp both enforced and passing). Includes the
expected pipeline model-state churn (25 logs).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/weight_robustness_diagnostic.xlsx
+++ b/outputs/weight_robustness_diagnostic.xlsx
@@ -1031,10 +1031,10 @@
         <v>51.5</v>
       </c>
       <c r="D8" t="n">
-        <v>57.64</v>
+        <v>56.46</v>
       </c>
       <c r="E8" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1042,10 +1042,10 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>52.43</v>
+        <v>51.65</v>
       </c>
       <c r="H8" t="n">
-        <v>31.9</v>
+        <v>29.9</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -1053,10 +1053,10 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>54.18</v>
+        <v>53.24</v>
       </c>
       <c r="K8" t="n">
-        <v>36.3</v>
+        <v>33.9</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="M8" t="n">
-        <v>50.33</v>
+        <v>49.77</v>
       </c>
       <c r="N8" t="n">
-        <v>26.6</v>
+        <v>25.2</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1075,10 +1075,10 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>52.2</v>
+        <v>51.48</v>
       </c>
       <c r="Q8" t="n">
-        <v>31.3</v>
+        <v>29.5</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>

</xml_diff>